<commit_message>
Rotisserie Chicken Kit F2: ensamblado, gates G1-G9 y revisión adversarial (0 B · 3 M · 6 m, todo arreglado; TPHC corregido, pestañas reales, sin marcas)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/rotisserie-chicken-restaurant-business-plan/rotisserie-chicken-yield-costing-calculator.xlsx
+++ b/astro-site/public/dl/rotisserie-chicken-restaurant-business-plan/rotisserie-chicken-yield-costing-calculator.xlsx
@@ -2165,7 +2165,7 @@
       </c>
       <c r="L13" s="25" t="inlineStr">
         <is>
-          <t>Inca Kola or soda</t>
+          <t>Peruvian or other soda</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -2652,7 +2652,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>Inca Kola or soda, can or bottle (ea)</t>
+          <t>Peruvian or other soda, can or bottle (ea)</t>
         </is>
       </c>
       <c r="B25" s="31" t="n">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="L27" s="3" t="str">
         <f>L13</f>
-        <v>Inca Kola or soda</v>
+        <v>Peruvian or other soda</v>
       </c>
     </row>
     <row r="28">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="L38" s="3" t="str">
         <f>L13</f>
-        <v>Inca Kola or soda</v>
+        <v>Peruvian or other soda</v>
       </c>
     </row>
     <row r="39">
@@ -3628,7 +3628,7 @@
     <row r="8" ht="75" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>3. Food safety. Probe the thickest part of the thigh: 165 °F is the Food Code cook temperature for poultry. In the heated display, hold at 135 °F or above, and check your county's rules for hot holding and for time as a public health control, which usually need a written procedure and a time mark on every load. Leftover you want to reuse is cooled from 135 to 70 °F within 2 hours and to 41 °F within 6 hours in total, and reheated to 165 °F for hot holding. Local rules vary: ask your health department.</t>
+          <t>3. Food safety. Probe the thickest part of the thigh: 165 °F is the Food Code cook temperature for poultry. In the heated display, hold at 135 °F or above, and check your county's rules for hot holding and for time as a public health control, which usually need a written procedure and a time mark on every load (under that control, birds are thrown out at 4 hours, never cooled). Leftover you want to reuse is cooled from 135 to 70 °F within 2 hours and to 41 °F within 6 hours in total, and reheated to 165 °F for hot holding. Local rules vary: ask your health department.</t>
         </is>
       </c>
     </row>

</xml_diff>